<commit_message>
test: round-3 GO retest after cookies, Redis limits, metrics, refunds
Merge auth cookie/refresh, wider rate limits, Prometheus, refunds.
Extend security suite; API 155/155 passed. Update GO report + Excel
checklists (UI + GO checklist workbooks).

Co-authored-by: manojkparija <manojkparija@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/qa/GAADIIQ_UI_Test_Results.xlsx
+++ b/docs/qa/GAADIIQ_UI_Test_Results.xlsx
@@ -526,7 +526,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-07-15 15:40 UTC</t>
+          <t>Generated: 2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -1528,7 +1528,7 @@
       <c r="I2" s="10" t="inlineStr"/>
       <c r="J2" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -1576,7 +1576,7 @@
       <c r="I3" s="10" t="inlineStr"/>
       <c r="J3" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -1624,7 +1624,7 @@
       <c r="I4" s="10" t="inlineStr"/>
       <c r="J4" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -1672,7 +1672,7 @@
       <c r="I5" s="10" t="inlineStr"/>
       <c r="J5" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -1720,7 +1720,7 @@
       <c r="I6" s="10" t="inlineStr"/>
       <c r="J6" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -1768,7 +1768,7 @@
       <c r="I7" s="10" t="inlineStr"/>
       <c r="J7" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -1816,7 +1816,7 @@
       <c r="I8" s="10" t="inlineStr"/>
       <c r="J8" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -1864,7 +1864,7 @@
       <c r="I9" s="10" t="inlineStr"/>
       <c r="J9" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -1912,7 +1912,7 @@
       <c r="I10" s="10" t="inlineStr"/>
       <c r="J10" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -1960,7 +1960,7 @@
       <c r="I11" s="10" t="inlineStr"/>
       <c r="J11" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -2008,7 +2008,7 @@
       <c r="I12" s="10" t="inlineStr"/>
       <c r="J12" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -2056,7 +2056,7 @@
       <c r="I13" s="10" t="inlineStr"/>
       <c r="J13" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -2104,7 +2104,7 @@
       <c r="I14" s="10" t="inlineStr"/>
       <c r="J14" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -2152,7 +2152,7 @@
       <c r="I15" s="10" t="inlineStr"/>
       <c r="J15" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -2200,7 +2200,7 @@
       <c r="I16" s="10" t="inlineStr"/>
       <c r="J16" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -2248,7 +2248,7 @@
       <c r="I17" s="10" t="inlineStr"/>
       <c r="J17" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -2296,7 +2296,7 @@
       <c r="I18" s="10" t="inlineStr"/>
       <c r="J18" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -2344,7 +2344,7 @@
       <c r="I19" s="10" t="inlineStr"/>
       <c r="J19" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -2392,7 +2392,7 @@
       <c r="I20" s="10" t="inlineStr"/>
       <c r="J20" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -2440,7 +2440,7 @@
       <c r="I21" s="10" t="inlineStr"/>
       <c r="J21" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -2488,7 +2488,7 @@
       <c r="I22" s="10" t="inlineStr"/>
       <c r="J22" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -2536,7 +2536,7 @@
       <c r="I23" s="10" t="inlineStr"/>
       <c r="J23" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -2584,7 +2584,7 @@
       <c r="I24" s="10" t="inlineStr"/>
       <c r="J24" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -2632,7 +2632,7 @@
       <c r="I25" s="10" t="inlineStr"/>
       <c r="J25" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -2680,7 +2680,7 @@
       <c r="I26" s="10" t="inlineStr"/>
       <c r="J26" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -2728,7 +2728,7 @@
       <c r="I27" s="10" t="inlineStr"/>
       <c r="J27" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -2776,7 +2776,7 @@
       <c r="I28" s="10" t="inlineStr"/>
       <c r="J28" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -2824,7 +2824,7 @@
       <c r="I29" s="10" t="inlineStr"/>
       <c r="J29" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -2872,7 +2872,7 @@
       <c r="I30" s="10" t="inlineStr"/>
       <c r="J30" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -2920,7 +2920,7 @@
       <c r="I31" s="10" t="inlineStr"/>
       <c r="J31" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -2968,7 +2968,7 @@
       <c r="I32" s="10" t="inlineStr"/>
       <c r="J32" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -3016,7 +3016,7 @@
       <c r="I33" s="10" t="inlineStr"/>
       <c r="J33" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -3064,7 +3064,7 @@
       <c r="I34" s="10" t="inlineStr"/>
       <c r="J34" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -3112,7 +3112,7 @@
       <c r="I35" s="10" t="inlineStr"/>
       <c r="J35" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -3160,7 +3160,7 @@
       <c r="I36" s="10" t="inlineStr"/>
       <c r="J36" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -3287,7 +3287,7 @@
       <c r="I2" s="10" t="inlineStr"/>
       <c r="J2" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -3335,7 +3335,7 @@
       <c r="I3" s="10" t="inlineStr"/>
       <c r="J3" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -3383,7 +3383,7 @@
       <c r="I4" s="10" t="inlineStr"/>
       <c r="J4" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -3431,7 +3431,7 @@
       <c r="I5" s="10" t="inlineStr"/>
       <c r="J5" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -3479,7 +3479,7 @@
       <c r="I6" s="10" t="inlineStr"/>
       <c r="J6" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -3527,7 +3527,7 @@
       <c r="I7" s="10" t="inlineStr"/>
       <c r="J7" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -3575,7 +3575,7 @@
       <c r="I8" s="10" t="inlineStr"/>
       <c r="J8" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -3623,7 +3623,7 @@
       <c r="I9" s="10" t="inlineStr"/>
       <c r="J9" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -3671,7 +3671,7 @@
       <c r="I10" s="10" t="inlineStr"/>
       <c r="J10" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -3719,7 +3719,7 @@
       <c r="I11" s="10" t="inlineStr"/>
       <c r="J11" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -3767,7 +3767,7 @@
       <c r="I12" s="10" t="inlineStr"/>
       <c r="J12" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -3815,7 +3815,7 @@
       <c r="I13" s="10" t="inlineStr"/>
       <c r="J13" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -3863,7 +3863,7 @@
       <c r="I14" s="10" t="inlineStr"/>
       <c r="J14" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -3911,7 +3911,7 @@
       <c r="I15" s="10" t="inlineStr"/>
       <c r="J15" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -3959,7 +3959,7 @@
       <c r="I16" s="10" t="inlineStr"/>
       <c r="J16" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -4007,7 +4007,7 @@
       <c r="I17" s="10" t="inlineStr"/>
       <c r="J17" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -4055,7 +4055,7 @@
       <c r="I18" s="10" t="inlineStr"/>
       <c r="J18" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -4103,7 +4103,7 @@
       <c r="I19" s="10" t="inlineStr"/>
       <c r="J19" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -4151,7 +4151,7 @@
       <c r="I20" s="10" t="inlineStr"/>
       <c r="J20" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -4199,7 +4199,7 @@
       <c r="I21" s="10" t="inlineStr"/>
       <c r="J21" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -4247,7 +4247,7 @@
       <c r="I22" s="10" t="inlineStr"/>
       <c r="J22" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -4295,7 +4295,7 @@
       <c r="I23" s="10" t="inlineStr"/>
       <c r="J23" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -4343,7 +4343,7 @@
       <c r="I24" s="10" t="inlineStr"/>
       <c r="J24" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -4391,7 +4391,7 @@
       <c r="I25" s="10" t="inlineStr"/>
       <c r="J25" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -4439,7 +4439,7 @@
       <c r="I26" s="10" t="inlineStr"/>
       <c r="J26" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -4487,7 +4487,7 @@
       <c r="I27" s="10" t="inlineStr"/>
       <c r="J27" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -4535,7 +4535,7 @@
       <c r="I28" s="10" t="inlineStr"/>
       <c r="J28" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -4583,7 +4583,7 @@
       <c r="I29" s="10" t="inlineStr"/>
       <c r="J29" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -4699,7 +4699,7 @@
       </c>
       <c r="G2" s="10" t="inlineStr">
         <is>
-          <t>Started pid=13635 status=200</t>
+          <t>Already running (200)</t>
         </is>
       </c>
       <c r="H2" s="10" t="inlineStr">
@@ -4710,7 +4710,7 @@
       <c r="I2" s="10" t="inlineStr"/>
       <c r="J2" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -4758,7 +4758,7 @@
       <c r="I3" s="10" t="inlineStr"/>
       <c r="J3" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -4806,7 +4806,7 @@
       <c r="I4" s="10" t="inlineStr"/>
       <c r="J4" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -4854,7 +4854,7 @@
       <c r="I5" s="10" t="inlineStr"/>
       <c r="J5" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -4902,7 +4902,7 @@
       <c r="I6" s="10" t="inlineStr"/>
       <c r="J6" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -4950,7 +4950,7 @@
       <c r="I7" s="10" t="inlineStr"/>
       <c r="J7" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -4998,7 +4998,7 @@
       <c r="I8" s="10" t="inlineStr"/>
       <c r="J8" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -5046,7 +5046,7 @@
       <c r="I9" s="10" t="inlineStr"/>
       <c r="J9" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -5094,7 +5094,7 @@
       <c r="I10" s="10" t="inlineStr"/>
       <c r="J10" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -5142,7 +5142,7 @@
       <c r="I11" s="10" t="inlineStr"/>
       <c r="J11" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -5190,7 +5190,7 @@
       <c r="I12" s="10" t="inlineStr"/>
       <c r="J12" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -5238,7 +5238,7 @@
       <c r="I13" s="10" t="inlineStr"/>
       <c r="J13" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -5286,7 +5286,7 @@
       <c r="I14" s="10" t="inlineStr"/>
       <c r="J14" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -5334,7 +5334,7 @@
       <c r="I15" s="10" t="inlineStr"/>
       <c r="J15" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -5386,7 +5386,7 @@
       </c>
       <c r="J16" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -5434,7 +5434,7 @@
       <c r="I17" s="10" t="inlineStr"/>
       <c r="J17" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -5482,7 +5482,7 @@
       <c r="I18" s="10" t="inlineStr"/>
       <c r="J18" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -5530,7 +5530,7 @@
       <c r="I19" s="10" t="inlineStr"/>
       <c r="J19" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -5657,7 +5657,7 @@
       <c r="I2" s="10" t="inlineStr"/>
       <c r="J2" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -5705,7 +5705,7 @@
       <c r="I3" s="10" t="inlineStr"/>
       <c r="J3" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -5753,7 +5753,7 @@
       <c r="I4" s="10" t="inlineStr"/>
       <c r="J4" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -5801,7 +5801,7 @@
       <c r="I5" s="10" t="inlineStr"/>
       <c r="J5" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -5849,7 +5849,7 @@
       <c r="I6" s="10" t="inlineStr"/>
       <c r="J6" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -5897,7 +5897,7 @@
       <c r="I7" s="10" t="inlineStr"/>
       <c r="J7" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -5945,7 +5945,7 @@
       <c r="I8" s="10" t="inlineStr"/>
       <c r="J8" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -5993,7 +5993,7 @@
       <c r="I9" s="10" t="inlineStr"/>
       <c r="J9" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -6041,7 +6041,7 @@
       <c r="I10" s="10" t="inlineStr"/>
       <c r="J10" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -6089,7 +6089,7 @@
       <c r="I11" s="10" t="inlineStr"/>
       <c r="J11" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -6137,7 +6137,7 @@
       <c r="I12" s="10" t="inlineStr"/>
       <c r="J12" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -6185,7 +6185,7 @@
       <c r="I13" s="10" t="inlineStr"/>
       <c r="J13" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -6233,7 +6233,7 @@
       <c r="I14" s="10" t="inlineStr"/>
       <c r="J14" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -6281,7 +6281,7 @@
       <c r="I15" s="10" t="inlineStr"/>
       <c r="J15" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -6329,7 +6329,7 @@
       <c r="I16" s="10" t="inlineStr"/>
       <c r="J16" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -6377,7 +6377,7 @@
       <c r="I17" s="10" t="inlineStr"/>
       <c r="J17" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -6425,7 +6425,7 @@
       <c r="I18" s="10" t="inlineStr"/>
       <c r="J18" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -6552,7 +6552,7 @@
       <c r="I2" s="10" t="inlineStr"/>
       <c r="J2" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -6600,7 +6600,7 @@
       <c r="I3" s="10" t="inlineStr"/>
       <c r="J3" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -6648,7 +6648,7 @@
       <c r="I4" s="10" t="inlineStr"/>
       <c r="J4" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -6696,7 +6696,7 @@
       <c r="I5" s="10" t="inlineStr"/>
       <c r="J5" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -6744,7 +6744,7 @@
       <c r="I6" s="10" t="inlineStr"/>
       <c r="J6" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -6792,7 +6792,7 @@
       <c r="I7" s="10" t="inlineStr"/>
       <c r="J7" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -6840,7 +6840,7 @@
       <c r="I8" s="10" t="inlineStr"/>
       <c r="J8" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -6888,7 +6888,7 @@
       <c r="I9" s="10" t="inlineStr"/>
       <c r="J9" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -6936,7 +6936,7 @@
       <c r="I10" s="10" t="inlineStr"/>
       <c r="J10" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -6984,7 +6984,7 @@
       <c r="I11" s="10" t="inlineStr"/>
       <c r="J11" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -7032,7 +7032,7 @@
       <c r="I12" s="10" t="inlineStr"/>
       <c r="J12" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -7080,7 +7080,7 @@
       <c r="I13" s="10" t="inlineStr"/>
       <c r="J13" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -7128,7 +7128,7 @@
       <c r="I14" s="10" t="inlineStr"/>
       <c r="J14" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -7176,7 +7176,7 @@
       <c r="I15" s="10" t="inlineStr"/>
       <c r="J15" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -7224,7 +7224,7 @@
       <c r="I16" s="10" t="inlineStr"/>
       <c r="J16" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -7272,7 +7272,7 @@
       <c r="I17" s="10" t="inlineStr"/>
       <c r="J17" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -7320,7 +7320,7 @@
       <c r="I18" s="10" t="inlineStr"/>
       <c r="J18" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -7368,7 +7368,7 @@
       <c r="I19" s="10" t="inlineStr"/>
       <c r="J19" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -7416,7 +7416,7 @@
       <c r="I20" s="10" t="inlineStr"/>
       <c r="J20" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -7464,7 +7464,7 @@
       <c r="I21" s="10" t="inlineStr"/>
       <c r="J21" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -7512,7 +7512,7 @@
       <c r="I22" s="10" t="inlineStr"/>
       <c r="J22" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -7560,7 +7560,7 @@
       <c r="I23" s="10" t="inlineStr"/>
       <c r="J23" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -7608,7 +7608,7 @@
       <c r="I24" s="10" t="inlineStr"/>
       <c r="J24" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -7656,7 +7656,7 @@
       <c r="I25" s="10" t="inlineStr"/>
       <c r="J25" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -7704,7 +7704,7 @@
       <c r="I26" s="10" t="inlineStr"/>
       <c r="J26" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -7752,7 +7752,7 @@
       <c r="I27" s="10" t="inlineStr"/>
       <c r="J27" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -7800,7 +7800,7 @@
       <c r="I28" s="10" t="inlineStr"/>
       <c r="J28" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -7848,7 +7848,7 @@
       <c r="I29" s="10" t="inlineStr"/>
       <c r="J29" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -7896,7 +7896,7 @@
       <c r="I30" s="10" t="inlineStr"/>
       <c r="J30" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -7944,7 +7944,7 @@
       <c r="I31" s="10" t="inlineStr"/>
       <c r="J31" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -7992,7 +7992,7 @@
       <c r="I32" s="10" t="inlineStr"/>
       <c r="J32" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -8040,7 +8040,7 @@
       <c r="I33" s="10" t="inlineStr"/>
       <c r="J33" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -8088,7 +8088,7 @@
       <c r="I34" s="10" t="inlineStr"/>
       <c r="J34" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -8136,7 +8136,7 @@
       <c r="I35" s="10" t="inlineStr"/>
       <c r="J35" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -8184,7 +8184,7 @@
       <c r="I36" s="10" t="inlineStr"/>
       <c r="J36" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -8232,7 +8232,7 @@
       <c r="I37" s="10" t="inlineStr"/>
       <c r="J37" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -8280,7 +8280,7 @@
       <c r="I38" s="10" t="inlineStr"/>
       <c r="J38" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -8328,7 +8328,7 @@
       <c r="I39" s="10" t="inlineStr"/>
       <c r="J39" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -8376,7 +8376,7 @@
       <c r="I40" s="10" t="inlineStr"/>
       <c r="J40" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -8424,7 +8424,7 @@
       <c r="I41" s="10" t="inlineStr"/>
       <c r="J41" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -8472,7 +8472,7 @@
       <c r="I42" s="10" t="inlineStr"/>
       <c r="J42" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -8520,7 +8520,7 @@
       <c r="I43" s="10" t="inlineStr"/>
       <c r="J43" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -8568,7 +8568,7 @@
       <c r="I44" s="10" t="inlineStr"/>
       <c r="J44" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -8616,7 +8616,7 @@
       <c r="I45" s="10" t="inlineStr"/>
       <c r="J45" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -8664,7 +8664,7 @@
       <c r="I46" s="10" t="inlineStr"/>
       <c r="J46" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -8712,7 +8712,7 @@
       <c r="I47" s="10" t="inlineStr"/>
       <c r="J47" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -8760,7 +8760,7 @@
       <c r="I48" s="10" t="inlineStr"/>
       <c r="J48" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -8808,7 +8808,7 @@
       <c r="I49" s="10" t="inlineStr"/>
       <c r="J49" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -8856,7 +8856,7 @@
       <c r="I50" s="10" t="inlineStr"/>
       <c r="J50" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -8904,7 +8904,7 @@
       <c r="I51" s="10" t="inlineStr"/>
       <c r="J51" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -8952,7 +8952,7 @@
       <c r="I52" s="10" t="inlineStr"/>
       <c r="J52" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -9000,7 +9000,7 @@
       <c r="I53" s="10" t="inlineStr"/>
       <c r="J53" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -9048,7 +9048,7 @@
       <c r="I54" s="10" t="inlineStr"/>
       <c r="J54" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -9096,7 +9096,7 @@
       <c r="I55" s="10" t="inlineStr"/>
       <c r="J55" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -9144,7 +9144,7 @@
       <c r="I56" s="10" t="inlineStr"/>
       <c r="J56" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -9192,7 +9192,7 @@
       <c r="I57" s="10" t="inlineStr"/>
       <c r="J57" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -9240,7 +9240,7 @@
       <c r="I58" s="10" t="inlineStr"/>
       <c r="J58" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -9288,7 +9288,7 @@
       <c r="I59" s="10" t="inlineStr"/>
       <c r="J59" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -9336,7 +9336,7 @@
       <c r="I60" s="10" t="inlineStr"/>
       <c r="J60" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -9384,7 +9384,7 @@
       <c r="I61" s="10" t="inlineStr"/>
       <c r="J61" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -9432,7 +9432,7 @@
       <c r="I62" s="10" t="inlineStr"/>
       <c r="J62" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -9480,7 +9480,7 @@
       <c r="I63" s="10" t="inlineStr"/>
       <c r="J63" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -9528,7 +9528,7 @@
       <c r="I64" s="10" t="inlineStr"/>
       <c r="J64" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -9565,7 +9565,7 @@
       </c>
       <c r="G65" s="10" t="inlineStr">
         <is>
-          <t>Started pid=13635 status=200</t>
+          <t>Already running (200)</t>
         </is>
       </c>
       <c r="H65" s="10" t="inlineStr">
@@ -9576,7 +9576,7 @@
       <c r="I65" s="10" t="inlineStr"/>
       <c r="J65" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -9624,7 +9624,7 @@
       <c r="I66" s="10" t="inlineStr"/>
       <c r="J66" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -9672,7 +9672,7 @@
       <c r="I67" s="10" t="inlineStr"/>
       <c r="J67" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -9720,7 +9720,7 @@
       <c r="I68" s="10" t="inlineStr"/>
       <c r="J68" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -9768,7 +9768,7 @@
       <c r="I69" s="10" t="inlineStr"/>
       <c r="J69" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -9816,7 +9816,7 @@
       <c r="I70" s="10" t="inlineStr"/>
       <c r="J70" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -9864,7 +9864,7 @@
       <c r="I71" s="10" t="inlineStr"/>
       <c r="J71" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -9912,7 +9912,7 @@
       <c r="I72" s="10" t="inlineStr"/>
       <c r="J72" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -9960,7 +9960,7 @@
       <c r="I73" s="10" t="inlineStr"/>
       <c r="J73" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -10008,7 +10008,7 @@
       <c r="I74" s="10" t="inlineStr"/>
       <c r="J74" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -10056,7 +10056,7 @@
       <c r="I75" s="10" t="inlineStr"/>
       <c r="J75" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -10104,7 +10104,7 @@
       <c r="I76" s="10" t="inlineStr"/>
       <c r="J76" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -10152,7 +10152,7 @@
       <c r="I77" s="10" t="inlineStr"/>
       <c r="J77" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -10200,7 +10200,7 @@
       <c r="I78" s="10" t="inlineStr"/>
       <c r="J78" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -10252,7 +10252,7 @@
       </c>
       <c r="J79" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -10300,7 +10300,7 @@
       <c r="I80" s="10" t="inlineStr"/>
       <c r="J80" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -10348,7 +10348,7 @@
       <c r="I81" s="10" t="inlineStr"/>
       <c r="J81" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -10396,7 +10396,7 @@
       <c r="I82" s="10" t="inlineStr"/>
       <c r="J82" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -10444,7 +10444,7 @@
       <c r="I83" s="10" t="inlineStr"/>
       <c r="J83" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -10492,7 +10492,7 @@
       <c r="I84" s="10" t="inlineStr"/>
       <c r="J84" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -10540,7 +10540,7 @@
       <c r="I85" s="10" t="inlineStr"/>
       <c r="J85" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -10588,7 +10588,7 @@
       <c r="I86" s="10" t="inlineStr"/>
       <c r="J86" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -10636,7 +10636,7 @@
       <c r="I87" s="10" t="inlineStr"/>
       <c r="J87" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -10684,7 +10684,7 @@
       <c r="I88" s="10" t="inlineStr"/>
       <c r="J88" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -10732,7 +10732,7 @@
       <c r="I89" s="10" t="inlineStr"/>
       <c r="J89" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -10780,7 +10780,7 @@
       <c r="I90" s="10" t="inlineStr"/>
       <c r="J90" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -10828,7 +10828,7 @@
       <c r="I91" s="10" t="inlineStr"/>
       <c r="J91" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -10876,7 +10876,7 @@
       <c r="I92" s="10" t="inlineStr"/>
       <c r="J92" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -10924,7 +10924,7 @@
       <c r="I93" s="10" t="inlineStr"/>
       <c r="J93" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -10972,7 +10972,7 @@
       <c r="I94" s="10" t="inlineStr"/>
       <c r="J94" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -11020,7 +11020,7 @@
       <c r="I95" s="10" t="inlineStr"/>
       <c r="J95" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -11068,7 +11068,7 @@
       <c r="I96" s="10" t="inlineStr"/>
       <c r="J96" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -11116,7 +11116,7 @@
       <c r="I97" s="10" t="inlineStr"/>
       <c r="J97" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -11164,7 +11164,7 @@
       <c r="I98" s="10" t="inlineStr"/>
       <c r="J98" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>
@@ -11212,7 +11212,7 @@
       <c r="I99" s="10" t="inlineStr"/>
       <c r="J99" s="10" t="inlineStr">
         <is>
-          <t>2026-07-15 15:40 UTC</t>
+          <t>2026-07-15 15:59 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>